<commit_message>
merging folders and such
</commit_message>
<xml_diff>
--- a/Research Logs/Research Log - Dave.xlsx
+++ b/Research Logs/Research Log - Dave.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="29628"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="6" rupBuild="30228"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\drdax\Desktop\work related\Weltec\2026\T1\Capstone\Week logbook changes\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://w2shared-my.sharepoint.com/personal/dave_sushames01_student_wandw_ac_nz/Documents/Documents/Capstone/Research Logs/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{AF0BDED7-A538-4982-BD37-86F9ACE43960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="23" documentId="13_ncr:1_{AF0BDED7-A538-4982-BD37-86F9ACE43960}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{14C8CA4B-C0CD-4179-997A-E9F86FF0C307}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="7200" yWindow="2595" windowWidth="21600" windowHeight="11385" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Research template" sheetId="1" r:id="rId1"/>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="9" uniqueCount="9">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="17" uniqueCount="17">
   <si>
     <t>Date</t>
   </si>
@@ -87,13 +87,37 @@
       <t xml:space="preserve"> edit D2 and D3 as they are automatic calculations</t>
     </r>
   </si>
+  <si>
+    <t>Searching</t>
+  </si>
+  <si>
+    <t>Google</t>
+  </si>
+  <si>
+    <t>Information on what happens when a PC is booted with two video cards</t>
+  </si>
+  <si>
+    <t>7 sources found and briefly examined</t>
+  </si>
+  <si>
+    <t>As above</t>
+  </si>
+  <si>
+    <t>Reading</t>
+  </si>
+  <si>
+    <t>https://forums.anandtech.com/threads/can-you-choose-which-gpu-to-use-as-primary.2466295/#post-38083422</t>
+  </si>
+  <si>
+    <t xml:space="preserve">Seems that it requires BIOS </t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
   <numFmts count="1">
-    <numFmt numFmtId="165" formatCode="d/mm/yy;@"/>
+    <numFmt numFmtId="164" formatCode="d/mm/yy;@"/>
   </numFmts>
   <fonts count="3" x14ac:knownFonts="1">
     <font>
@@ -153,10 +177,10 @@
       <alignment wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment horizontal="left" vertical="top"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1"/>
@@ -176,6 +200,10 @@
     </ext>
   </extLst>
 </styleSheet>
+</file>
+
+<file path=xl/persons/person.xml><?xml version="1.0" encoding="utf-8"?>
+<personList xmlns="http://schemas.microsoft.com/office/spreadsheetml/2018/threadedcomments" xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main"/>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -457,7 +485,7 @@
         <v>3</v>
       </c>
       <c r="D2" s="5">
-        <f>ROUNDDOWN(SUM(C6:C500)/60,0)</f>
+        <f>ROUNDDOWN(SUM(C7:C500)/60,0)</f>
         <v>0</v>
       </c>
       <c r="E2" t="s">
@@ -469,8 +497,8 @@
         <v>4</v>
       </c>
       <c r="D3" s="5">
-        <f>ROUND(MOD(SUM(C6:C500),60),0)</f>
-        <v>0</v>
+        <f>ROUND(MOD(SUM(C7:C500),60),0)</f>
+        <v>15</v>
       </c>
     </row>
     <row r="5" spans="2:7" x14ac:dyDescent="0.25">
@@ -493,9 +521,45 @@
         <v>6</v>
       </c>
     </row>
+    <row r="7" spans="2:7" x14ac:dyDescent="0.25">
+      <c r="B7" s="3">
+        <v>46234</v>
+      </c>
+      <c r="C7">
+        <v>10</v>
+      </c>
+      <c r="D7" t="s">
+        <v>9</v>
+      </c>
+      <c r="E7" t="s">
+        <v>11</v>
+      </c>
+      <c r="F7" t="s">
+        <v>12</v>
+      </c>
+      <c r="G7" t="s">
+        <v>10</v>
+      </c>
+    </row>
     <row r="8" spans="2:7" x14ac:dyDescent="0.25">
-      <c r="F8" s="1"/>
-      <c r="G8" s="1"/>
+      <c r="B8" s="3">
+        <v>46234</v>
+      </c>
+      <c r="C8">
+        <v>5</v>
+      </c>
+      <c r="D8" t="s">
+        <v>14</v>
+      </c>
+      <c r="E8" t="s">
+        <v>13</v>
+      </c>
+      <c r="F8" s="1" t="s">
+        <v>16</v>
+      </c>
+      <c r="G8" s="1" t="s">
+        <v>15</v>
+      </c>
     </row>
     <row r="9" spans="2:7" x14ac:dyDescent="0.25">
       <c r="F9" s="1"/>

</xml_diff>